<commit_message>
docs: classify competitor services for integration
</commit_message>
<xml_diff>
--- a/outputs/quantum-company-agent-monitor-20260904/中国量子公司传统服务与Agent服务监控清单-2026-09-04.xlsx
+++ b/outputs/quantum-company-agent-monitor-20260904/中国量子公司传统服务与Agent服务监控清单-2026-09-04.xlsx
@@ -2,10 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="Ra705c1973f9d4529"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="监控总表" sheetId="2" r:id="Rfa37567376f24910"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent重点对象" sheetId="3" r:id="Ref888b0428084e1b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="口径与更新" sheetId="4" r:id="R21cfb60c11e94fb9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="R76e8ef7a9b2c4ffc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="监控总表" sheetId="2" r:id="R989a299ec82e4236"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent重点对象" sheetId="3" r:id="R349994350fb44543"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="口径与更新" sheetId="4" r:id="R35fafbe6d1e0400a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="服务能力清单" sheetId="5" r:id="R61ec44a009c84189"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20,7 +21,7 @@
     <x:numFmt numFmtId="200" formatCode="0"/>
     <x:numFmt numFmtId="201" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
-  <x:fonts count="8">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -66,8 +67,25 @@
       <x:color rgb="FF163A5F"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="16"/>
+      <x:color rgb="FF17365D"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF666666"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FF222222"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -82,6 +100,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFE8EFF6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -186,7 +209,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="55">
+  <x:cellXfs count="78">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -296,18 +319,71 @@
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="4">
+  <x:dxfs count="7">
     <x:dxf>
       <x:font>
         <x:b/>
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
       </x:fill>
@@ -318,8 +394,40 @@
         <x:color rgb="FF1F4E78"/>
       </x:font>
       <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDDEBF7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF7F6000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF595959"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE7E6E6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFDDEBF7"/>
+          <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -336,7 +444,7 @@
     </x:dxf>
     <x:dxf>
       <x:font>
-        <x:color rgb="FF595959"/>
+        <x:color rgb="FF666666"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
@@ -388,6 +496,27 @@
     <x:tableColumn id="7" name="下一核验点"/>
     <x:tableColumn id="8" name="对OpenQuantum的意义"/>
     <x:tableColumn id="9" name="来源"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ServiceCapabilityTable" displayName="ServiceCapabilityTable" ref="A4:L34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:L34"/>
+  <x:tableColumns count="12">
+    <x:tableColumn id="1" name="序号"/>
+    <x:tableColumn id="2" name="公司"/>
+    <x:tableColumn id="3" name="技术路线"/>
+    <x:tableColumn id="4" name="领域算法和模拟器"/>
+    <x:tableColumn id="5" name="云平台和硬件接口"/>
+    <x:tableColumn id="6" name="低门槛 Agent 体验"/>
+    <x:tableColumn id="7" name="获取方式"/>
+    <x:tableColumn id="8" name="OpenQuantum 落点"/>
+    <x:tableColumn id="9" name="优先级"/>
+    <x:tableColumn id="10" name="下一步核验"/>
+    <x:tableColumn id="11" name="证据 URL"/>
+    <x:tableColumn id="12" name="最近核验"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -2801,7 +2930,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17fc8079d0b74402"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3867c53a297b4bc6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3046,7 +3175,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a35f6ebb7cf4ccc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0ae1d42fa2d4720"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3400,4 +3529,1283 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF2F75B5"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="7" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="19" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="32" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="34" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="34" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="30" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="10" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="38" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="42" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="12" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="55" t="str">
+        <x:v>30 家量子公司服务能力清单</x:v>
+      </x:c>
+      <x:c r="B1" s="55"/>
+      <x:c r="C1" s="55"/>
+      <x:c r="D1" s="55"/>
+      <x:c r="E1" s="55"/>
+      <x:c r="F1" s="55"/>
+      <x:c r="G1" s="55"/>
+      <x:c r="H1" s="55"/>
+      <x:c r="I1" s="55"/>
+      <x:c r="J1" s="55"/>
+      <x:c r="K1" s="55"/>
+      <x:c r="L1" s="55"/>
+    </x:row>
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2" s="57" t="str">
+        <x:v>只监控三类可产品化服务：领域算法和模拟器、云平台和硬件接口、低门槛 Agent 体验。每家公司一行，便于判断复用、接入或独立实现。</x:v>
+      </x:c>
+      <x:c r="B2" s="57"/>
+      <x:c r="C2" s="57"/>
+      <x:c r="D2" s="57"/>
+      <x:c r="E2" s="57"/>
+      <x:c r="F2" s="57"/>
+      <x:c r="G2" s="57"/>
+      <x:c r="H2" s="57"/>
+      <x:c r="I2" s="57"/>
+      <x:c r="J2" s="57"/>
+      <x:c r="K2" s="57"/>
+      <x:c r="L2" s="57"/>
+    </x:row>
+    <x:row r="3" ht="8" customHeight="1"/>
+    <x:row r="4" ht="34" customHeight="1">
+      <x:c r="A4" s="69" t="str">
+        <x:v>序号</x:v>
+      </x:c>
+      <x:c r="B4" s="70" t="str">
+        <x:v>公司</x:v>
+      </x:c>
+      <x:c r="C4" s="70" t="str">
+        <x:v>技术路线</x:v>
+      </x:c>
+      <x:c r="D4" s="70" t="str">
+        <x:v>领域算法和模拟器</x:v>
+      </x:c>
+      <x:c r="E4" s="70" t="str">
+        <x:v>云平台和硬件接口</x:v>
+      </x:c>
+      <x:c r="F4" s="70" t="str">
+        <x:v>低门槛 Agent 体验</x:v>
+      </x:c>
+      <x:c r="G4" s="70" t="str">
+        <x:v>获取方式</x:v>
+      </x:c>
+      <x:c r="H4" s="70" t="str">
+        <x:v>OpenQuantum 落点</x:v>
+      </x:c>
+      <x:c r="I4" s="70" t="str">
+        <x:v>优先级</x:v>
+      </x:c>
+      <x:c r="J4" s="70" t="str">
+        <x:v>下一步核验</x:v>
+      </x:c>
+      <x:c r="K4" s="70" t="str">
+        <x:v>证据 URL</x:v>
+      </x:c>
+      <x:c r="L4" s="71" t="str">
+        <x:v>最近核验</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="66" customHeight="1">
+      <x:c r="A5" s="75" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B5" s="75" t="str">
+        <x:v>中电信量子集团</x:v>
+      </x:c>
+      <x:c r="C5" s="75" t="str">
+        <x:v>超导</x:v>
+      </x:c>
+      <x:c r="D5" s="74" t="str">
+        <x:v>未确认独立开源算法或模拟器；公开服务以量子云和政企方案为主</x:v>
+      </x:c>
+      <x:c r="E5" s="74" t="str">
+        <x:v>天衍量子云、超导量子计算机、量子安全网络；第三方 FieldQKit 已能发现部分后端</x:v>
+      </x:c>
+      <x:c r="F5" s="74" t="str">
+        <x:v>集团有星辰智能体平台；未确认量子云工具已接入</x:v>
+      </x:c>
+      <x:c r="G5" s="74" t="str">
+        <x:v>官方接口接入</x:v>
+      </x:c>
+      <x:c r="H5" s="74" t="str">
+        <x:v>External API Adapter + Tool Provider</x:v>
+      </x:c>
+      <x:c r="I5" s="76" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="J5" s="74" t="str">
+        <x:v>核验天衍官方 SDK/API、鉴权、计费、提交/取消/结果合同</x:v>
+      </x:c>
+      <x:c r="K5" s="74" t="str">
+        <x:v>https://qc.zdxlz.com/
+https://www.chinatelecom.com.cn/ct/news/gdxw/167478.html
+https://github.com/FieldQuantum/fieldqkit</x:v>
+      </x:c>
+      <x:c r="L5" s="77" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="66" customHeight="1">
+      <x:c r="A6" s="75" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B6" s="75" t="str">
+        <x:v>国盾量子</x:v>
+      </x:c>
+      <x:c r="C6" s="75" t="str">
+        <x:v>超导</x:v>
+      </x:c>
+      <x:c r="D6" s="74" t="str">
+        <x:v>未确认独立开源算法或模拟器；公开软件面以云平台和系统工程为主</x:v>
+      </x:c>
+      <x:c r="E6" s="74" t="str">
+        <x:v>量子计算云、测控与制冷设备、量子安全设备；第三方 FieldQKit 已能发现部分后端</x:v>
+      </x:c>
+      <x:c r="F6" s="74" t="str">
+        <x:v>未见自然语言任务编排或公司自有 Agent</x:v>
+      </x:c>
+      <x:c r="G6" s="74" t="str">
+        <x:v>官方接口接入</x:v>
+      </x:c>
+      <x:c r="H6" s="74" t="str">
+        <x:v>External API Adapter + Tool Provider</x:v>
+      </x:c>
+      <x:c r="I6" s="76" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="J6" s="74" t="str">
+        <x:v>核验官方 SDK/API、云任务写入、回执、取消与真实 QPU 可用性</x:v>
+      </x:c>
+      <x:c r="K6" s="74" t="str">
+        <x:v>https://www.quantum-info.com/
+https://github.com/FieldQuantum/fieldqkit</x:v>
+      </x:c>
+      <x:c r="L6" s="77" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="66" customHeight="1">
+      <x:c r="A7" s="75" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B7" s="75" t="str">
+        <x:v>本源量子</x:v>
+      </x:c>
+      <x:c r="C7" s="75" t="str">
+        <x:v>超导</x:v>
+      </x:c>
+      <x:c r="D7" s="74" t="str">
+        <x:v>QPanda3、pyQPanda、QUBO 建模与求解、量子编程和模拟能力</x:v>
+      </x:c>
+      <x:c r="E7" s="74" t="str">
+        <x:v>量子云、超导 QPU、设备查询、采样/估计/批处理、任务状态/结果/取消</x:v>
+      </x:c>
+      <x:c r="F7" s="74" t="str">
+        <x:v>官方 QPanda3 Runtime MCP 提供 Agent 工具层；未形成完整终端用户 Agent</x:v>
+      </x:c>
+      <x:c r="G7" s="74" t="str">
+        <x:v>Apache-2.0 复用 + 官方接口接入</x:v>
+      </x:c>
+      <x:c r="H7" s="74" t="str">
+        <x:v>Harness MCP Client + Skill + Scientific Validator</x:v>
+      </x:c>
+      <x:c r="I7" s="76" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="J7" s="74" t="str">
+        <x:v>维护已接入能力；跟踪 MCP release、任务合同、计费和真实 QPU 稳定性</x:v>
+      </x:c>
+      <x:c r="K7" s="74" t="str">
+        <x:v>https://www.originqc.com.cn/
+https://github.com/OriginQ/qpanda3-runtime-mcp-server</x:v>
+      </x:c>
+      <x:c r="L7" s="77" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="66" customHeight="1">
+      <x:c r="A8" s="75" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B8" s="75" t="str">
+        <x:v>量旋科技</x:v>
+      </x:c>
+      <x:c r="C8" s="75" t="str">
+        <x:v>超导</x:v>
+      </x:c>
+      <x:c r="D8" s="74" t="str">
+        <x:v>教育实验、量子编程和在线实验软件；未确认可复用的官方公开仓库</x:v>
+      </x:c>
+      <x:c r="E8" s="74" t="str">
+        <x:v>核磁与超导整机、线上实验平台、测控和芯片工具</x:v>
+      </x:c>
+      <x:c r="F8" s="74" t="str">
+        <x:v>未见 MCP、Agent API 或端到端任务 Agent</x:v>
+      </x:c>
+      <x:c r="G8" s="74" t="str">
+        <x:v>公开行为独立实现；接口出现后接入</x:v>
+      </x:c>
+      <x:c r="H8" s="74" t="str">
+        <x:v>Skill + External API Adapter + Tool Provider</x:v>
+      </x:c>
+      <x:c r="I8" s="76" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="J8" s="74" t="str">
+        <x:v>核验 SpinQit/平台 API、许可证、Agent demo 和任务回执</x:v>
+      </x:c>
+      <x:c r="K8" s="74" t="str">
+        <x:v>https://www.spinq.com/zh/</x:v>
+      </x:c>
+      <x:c r="L8" s="77" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="66" customHeight="1">
+      <x:c r="A9" s="75" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B9" s="75" t="str">
+        <x:v>逻辑比特</x:v>
+      </x:c>
+      <x:c r="C9" s="75" t="str">
+        <x:v>超导</x:v>
+      </x:c>
+      <x:c r="D9" s="74" t="str">
+        <x:v>未确认独立开源算法库；主要价值是后端与任务服务</x:v>
+      </x:c>
+      <x:c r="E9" s="74" t="str">
+        <x:v>量子云 REST API/Token、超导 QPU、测控与射频系统</x:v>
+      </x:c>
+      <x:c r="F9" s="74" t="str">
+        <x:v>可作为 Agent 后端；未见公司自有 Agent 或官方 MCP</x:v>
+      </x:c>
+      <x:c r="G9" s="74" t="str">
+        <x:v>官方接口接入</x:v>
+      </x:c>
+      <x:c r="H9" s="74" t="str">
+        <x:v>External API Adapter + Tool Provider</x:v>
+      </x:c>
+      <x:c r="I9" s="76" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="J9" s="74" t="str">
+        <x:v>核验官方 API 合同、提交/取消/结果、限额与错误语义</x:v>
+      </x:c>
+      <x:c r="K9" s="74" t="str">
+        <x:v>https://logicalqubit.com/
+https://cloud.logicalqubit.com/landing/
+https://fieldquantum.github.io/fieldqkit/api/providers/</x:v>
+      </x:c>
+      <x:c r="L9" s="77" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="66" customHeight="1">
+      <x:c r="A10" s="75" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B10" s="75" t="str">
+        <x:v>相干科技</x:v>
+      </x:c>
+      <x:c r="C10" s="75" t="str">
+        <x:v>超导</x:v>
+      </x:c>
+      <x:c r="D10" s="74" t="str">
+        <x:v>量子测控、智能校准和控制软件方向；公开算法资产未确认</x:v>
+      </x:c>
+      <x:c r="E10" s="74" t="str">
+        <x:v>高密度测控电子学、云平台和整机方案</x:v>
+      </x:c>
+      <x:c r="F10" s="74" t="str">
+        <x:v>量子 AI 合作存在；未见公司自有 Agent 或 Agent API</x:v>
+      </x:c>
+      <x:c r="G10" s="74" t="str">
+        <x:v>接口接入 + 公开行为独立实现</x:v>
+      </x:c>
+      <x:c r="H10" s="74" t="str">
+        <x:v>Tool Provider + Scientific Validator</x:v>
+      </x:c>
+      <x:c r="I10" s="76" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="J10" s="74" t="str">
+        <x:v>核验测控协议、校准数据格式、可调用接口与权限边界</x:v>
+      </x:c>
+      <x:c r="K10" s="74" t="str">
+        <x:v>https://mp.weixin.qq.com/s/VqK81LJrWPYqd4UPI39S2g
+https://www.cww.net.cn/article?id=608430</x:v>
+      </x:c>
+      <x:c r="L10" s="77" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="66" customHeight="1">
+      <x:c r="A11" s="75" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B11" s="75" t="str">
+        <x:v>国基量子</x:v>
+      </x:c>
+      <x:c r="C11" s="75" t="str">
+        <x:v>超导</x:v>
+      </x:c>
+      <x:c r="D11" s="74" t="str">
+        <x:v>电子-量子混合计算与软件规划；未见公开 SDK/模拟器</x:v>
+      </x:c>
+      <x:c r="E11" s="74" t="str">
+        <x:v>国产超导整机、芯片制造、混合算力与云服务规划</x:v>
+      </x:c>
+      <x:c r="F11" s="74" t="str">
+        <x:v>未见公开任务型 Agent</x:v>
+      </x:c>
+      <x:c r="G11" s="74" t="str">
+        <x:v>公开行为独立实现；接口出现后接入</x:v>
+      </x:c>
+      <x:c r="H11" s="74" t="str">
+        <x:v>Skill + External API Adapter</x:v>
+      </x:c>
+      <x:c r="I11" s="76" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="J11" s="74" t="str">
+        <x:v>等待独立官网、云入口、SDK/API 和可验证任务案例</x:v>
+      </x:c>
+      <x:c r="K11" s="74" t="str">
+        <x:v>https://www.cetc.com.cn/
+https://news.ustc.edu.cn/info/1055/93916.htm</x:v>
+      </x:c>
+      <x:c r="L11" s="77" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="66" customHeight="1">
+      <x:c r="A12" s="75" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B12" s="75" t="str">
+        <x:v>矩量光启</x:v>
+      </x:c>
+      <x:c r="C12" s="75" t="str">
+        <x:v>超导</x:v>
+      </x:c>
+      <x:c r="D12" s="74" t="str">
+        <x:v>量子 EDA、芯片工艺和封装能力方向；未见公开软件</x:v>
+      </x:c>
+      <x:c r="E12" s="74" t="str">
+        <x:v>硅基超导芯片、整机、3D/TSV 工艺平台</x:v>
+      </x:c>
+      <x:c r="F12" s="74" t="str">
+        <x:v>未见云、API、SDK 或 Agent</x:v>
+      </x:c>
+      <x:c r="G12" s="74" t="str">
+        <x:v>仅监控</x:v>
+      </x:c>
+      <x:c r="H12" s="74" t="str">
+        <x:v>暂不接入</x:v>
+      </x:c>
+      <x:c r="I12" s="76" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="J12" s="74" t="str">
+        <x:v>等待产品文档、首个软件仓库或机器接口</x:v>
+      </x:c>
+      <x:c r="K12" s="74" t="str">
+        <x:v>https://www.sqcomputing.com/</x:v>
+      </x:c>
+      <x:c r="L12" s="77" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="66" customHeight="1">
+      <x:c r="A13" s="75" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B13" s="75" t="str">
+        <x:v>正元量子</x:v>
+      </x:c>
+      <x:c r="C13" s="75" t="str">
+        <x:v>超导</x:v>
+      </x:c>
+      <x:c r="D13" s="74" t="str">
+        <x:v>量子 EDA、控制软件和集成测控规划；未见公开实现</x:v>
+      </x:c>
+      <x:c r="E13" s="74" t="str">
+        <x:v>3D 同轴封装、耦合器芯片、参量放大器和测控部件</x:v>
+      </x:c>
+      <x:c r="F13" s="74" t="str">
+        <x:v>未见公开 Agent</x:v>
+      </x:c>
+      <x:c r="G13" s="74" t="str">
+        <x:v>公开行为独立实现；接口出现后接入</x:v>
+      </x:c>
+      <x:c r="H13" s="74" t="str">
+        <x:v>Skill + Tool Provider</x:v>
+      </x:c>
+      <x:c r="I13" s="76" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="J13" s="74" t="str">
+        <x:v>核验 EDA/控制软件发布、数据格式、SDK/API</x:v>
+      </x:c>
+      <x:c r="K13" s="74" t="str">
+        <x:v>https://mp.weixin.qq.com/s/VqK81LJrWPYqd4UPI39S2g</x:v>
+      </x:c>
+      <x:c r="L13" s="77" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="66" customHeight="1">
+      <x:c r="A14" s="75" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B14" s="75" t="str">
+        <x:v>华翊博奥（华翊量子）</x:v>
+      </x:c>
+      <x:c r="C14" s="75" t="str">
+        <x:v>离子阱</x:v>
+      </x:c>
+      <x:c r="D14" s="74" t="str">
+        <x:v>离子阱算法和行业应用探索；未确认公开模拟器</x:v>
+      </x:c>
+      <x:c r="E14" s="74" t="str">
+        <x:v>离子阱整机、激光稳频/测控部件、无极一号量子云</x:v>
+      </x:c>
+      <x:c r="F14" s="74" t="str">
+        <x:v>有量子 AI 平台合作；未见公司自有 Agent</x:v>
+      </x:c>
+      <x:c r="G14" s="74" t="str">
+        <x:v>官方接口接入</x:v>
+      </x:c>
+      <x:c r="H14" s="74" t="str">
+        <x:v>External API Adapter + Tool Provider</x:v>
+      </x:c>
+      <x:c r="I14" s="76" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="J14" s="74" t="str">
+        <x:v>核验云 SDK/API、任务合同、结果结构和量智工具化</x:v>
+      </x:c>
+      <x:c r="K14" s="74" t="str">
+        <x:v>https://www.hyqubit.com/
+https://www.hyqubit.com/newsinfo/8534506.html
+https://www.hyqubit.com/newsinfo/10836695.html</x:v>
+      </x:c>
+      <x:c r="L14" s="77" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="66" customHeight="1">
+      <x:c r="A15" s="75" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B15" s="75" t="str">
+        <x:v>幺正量子</x:v>
+      </x:c>
+      <x:c r="C15" s="75" t="str">
+        <x:v>离子阱</x:v>
+      </x:c>
+      <x:c r="D15" s="74" t="str">
+        <x:v>离子阱算法与材料、生医、安全等行业方案；未见公开算法仓库</x:v>
+      </x:c>
+      <x:c r="E15" s="74" t="str">
+        <x:v>QCCD 离子阱整机、部件和量子算力云</x:v>
+      </x:c>
+      <x:c r="F15" s="74" t="str">
+        <x:v>未见公司自有 Agent、MCP 或 Agent API</x:v>
+      </x:c>
+      <x:c r="G15" s="74" t="str">
+        <x:v>官方接口接入</x:v>
+      </x:c>
+      <x:c r="H15" s="74" t="str">
+        <x:v>External API Adapter + Tool Provider</x:v>
+      </x:c>
+      <x:c r="I15" s="76" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="J15" s="74" t="str">
+        <x:v>核验量子云开放方式、SDK/API、任务回执和取消能力</x:v>
+      </x:c>
+      <x:c r="K15" s="74" t="str">
+        <x:v>https://www.unitqc.com/
+https://www.unitqc.com/?c=1</x:v>
+      </x:c>
+      <x:c r="L15" s="77" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="66" customHeight="1">
+      <x:c r="A16" s="75" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B16" s="75" t="str">
+        <x:v>维刻量光</x:v>
+      </x:c>
+      <x:c r="C16" s="75" t="str">
+        <x:v>离子阱</x:v>
+      </x:c>
+      <x:c r="D16" s="74" t="str">
+        <x:v>离子阱控制软件、量子指令集和平台接口方向</x:v>
+      </x:c>
+      <x:c r="E16" s="74" t="str">
+        <x:v>QCCD 表面阱芯片 IDM、控制系统和平台接口</x:v>
+      </x:c>
+      <x:c r="F16" s="74" t="str">
+        <x:v>未见公开 Agent</x:v>
+      </x:c>
+      <x:c r="G16" s="74" t="str">
+        <x:v>接口接入 + 公开行为独立实现</x:v>
+      </x:c>
+      <x:c r="H16" s="74" t="str">
+        <x:v>Tool Provider + Skill</x:v>
+      </x:c>
+      <x:c r="I16" s="76" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="J16" s="74" t="str">
+        <x:v>核验指令集、SDK/API、控制协议和首个代码仓库</x:v>
+      </x:c>
+      <x:c r="K16" s="74" t="str">
+        <x:v>https://mp.weixin.qq.com/s/VqK81LJrWPYqd4UPI39S2g
+https://www.36kr.com/p/3805641110511367
+https://svtr.ai/orgs/weikeliangguang</x:v>
+      </x:c>
+      <x:c r="L16" s="77" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="66" customHeight="1">
+      <x:c r="A17" s="75" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B17" s="75" t="str">
+        <x:v>玉盘智能</x:v>
+      </x:c>
+      <x:c r="C17" s="75" t="str">
+        <x:v>离子阱</x:v>
+      </x:c>
+      <x:c r="D17" s="74" t="str">
+        <x:v>AI 驱动量子控制、自优化/自学习控制和低时延调度</x:v>
+      </x:c>
+      <x:c r="E17" s="74" t="str">
+        <x:v>控制芯片、MQPU 和 AI-QCaaS 路线</x:v>
+      </x:c>
+      <x:c r="F17" s="74" t="str">
+        <x:v>当前是控制系统智能化，不是用户任务 Agent</x:v>
+      </x:c>
+      <x:c r="G17" s="74" t="str">
+        <x:v>公开行为独立实现；未来官方接口接入</x:v>
+      </x:c>
+      <x:c r="H17" s="74" t="str">
+        <x:v>Tool Provider + Scientific Validator</x:v>
+      </x:c>
+      <x:c r="I17" s="76" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="J17" s="74" t="str">
+        <x:v>核验 MQuest API、控制闭环证据、权限和真实芯片结果</x:v>
+      </x:c>
+      <x:c r="K17" s="74" t="str">
+        <x:v>https://www.moonquest.cn/</x:v>
+      </x:c>
+      <x:c r="L17" s="77" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="66" customHeight="1">
+      <x:c r="A18" s="75" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B18" s="75" t="str">
+        <x:v>中科酷原</x:v>
+      </x:c>
+      <x:c r="C18" s="75" t="str">
+        <x:v>中性原子</x:v>
+      </x:c>
+      <x:c r="D18" s="74" t="str">
+        <x:v>中性原子计算、优化及医药化工应用服务；未确认公开模拟器仓库</x:v>
+      </x:c>
+      <x:c r="E18" s="74" t="str">
+        <x:v>中性原子整机、测控/光学部件和汉原量子云</x:v>
+      </x:c>
+      <x:c r="F18" s="74" t="str">
+        <x:v>未见 Agent、MCP 或 Agent API</x:v>
+      </x:c>
+      <x:c r="G18" s="74" t="str">
+        <x:v>官方接口接入</x:v>
+      </x:c>
+      <x:c r="H18" s="74" t="str">
+        <x:v>External API Adapter + Tool Provider</x:v>
+      </x:c>
+      <x:c r="I18" s="76" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="J18" s="74" t="str">
+        <x:v>核验汉原云 API/SDK、任务结构、后端约束和结果证据</x:v>
+      </x:c>
+      <x:c r="K18" s="74" t="str">
+        <x:v>https://www.cascoldatom.com/</x:v>
+      </x:c>
+      <x:c r="L18" s="77" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="66" customHeight="1">
+      <x:c r="A19" s="75" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B19" s="75" t="str">
+        <x:v>QUANTier</x:v>
+      </x:c>
+      <x:c r="C19" s="75" t="str">
+        <x:v>中性原子</x:v>
+      </x:c>
+      <x:c r="D19" s="74" t="str">
+        <x:v>浏览器量子编程、图形化实验和中间件能力</x:v>
+      </x:c>
+      <x:c r="E19" s="74" t="str">
+        <x:v>量子云 SaaS、中性原子中间件与硬件接口</x:v>
+      </x:c>
+      <x:c r="F19" s="74" t="str">
+        <x:v>低门槛图形体验较强；未见任务型 Agent</x:v>
+      </x:c>
+      <x:c r="G19" s="74" t="str">
+        <x:v>公开行为独立实现；接口出现后接入</x:v>
+      </x:c>
+      <x:c r="H19" s="74" t="str">
+        <x:v>Client Plugin + Skill + External API Adapter</x:v>
+      </x:c>
+      <x:c r="I19" s="76" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="J19" s="74" t="str">
+        <x:v>核验开源计划、API/SDK、硬件接入合同和任务回执</x:v>
+      </x:c>
+      <x:c r="K19" s="74" t="str">
+        <x:v>https://quantier.io/
+https://quantier.io/home/</x:v>
+      </x:c>
+      <x:c r="L19" s="77" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="66" customHeight="1">
+      <x:c r="A20" s="75" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B20" s="75" t="str">
+        <x:v>两仪万象</x:v>
+      </x:c>
+      <x:c r="C20" s="75" t="str">
+        <x:v>中性原子</x:v>
+      </x:c>
+      <x:c r="D20" s="74" t="str">
+        <x:v>实验控制、数据分析和日常运维工作流；算法资产尚未公开</x:v>
+      </x:c>
+      <x:c r="E20" s="74" t="str">
+        <x:v>中性原子整机、测控系统、量子软件和云平台</x:v>
+      </x:c>
+      <x:c r="F20" s="74" t="str">
+        <x:v>量智开物明确研发智能体量子计算机，目标是可调用、可组合、可验证的实验工具</x:v>
+      </x:c>
+      <x:c r="G20" s="74" t="str">
+        <x:v>公开行为独立实现；官方接口出现后接入</x:v>
+      </x:c>
+      <x:c r="H20" s="74" t="str">
+        <x:v>Skill + Tool Provider + Scientific Validator</x:v>
+      </x:c>
+      <x:c r="I20" s="76" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="J20" s="74" t="str">
+        <x:v>跟踪首个可用 Agent、工具 schema、权限、实验闭环和来源链</x:v>
+      </x:c>
+      <x:c r="K20" s="74" t="str">
+        <x:v>https://atomtoinfinity.com/
+https://www.iqitek.com/</x:v>
+      </x:c>
+      <x:c r="L20" s="77" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="66" customHeight="1">
+      <x:c r="A21" s="75" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B21" s="75" t="str">
+        <x:v>中器无量</x:v>
+      </x:c>
+      <x:c r="C21" s="75" t="str">
+        <x:v>中性原子</x:v>
+      </x:c>
+      <x:c r="D21" s="74" t="str">
+        <x:v>行业优化与量子应用方向；未确认公开算法/模拟器</x:v>
+      </x:c>
+      <x:c r="E21" s="74" t="str">
+        <x:v>中性原子整机、万比特算力基础设施和运营商云合作</x:v>
+      </x:c>
+      <x:c r="F21" s="74" t="str">
+        <x:v>未见公司自有 Agent、SDK 或 MCP</x:v>
+      </x:c>
+      <x:c r="G21" s="74" t="str">
+        <x:v>官方接口接入</x:v>
+      </x:c>
+      <x:c r="H21" s="74" t="str">
+        <x:v>External API Adapter + Tool Provider</x:v>
+      </x:c>
+      <x:c r="I21" s="76" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="J21" s="74" t="str">
+        <x:v>核验移动云入口、API/SDK、资源调度和任务回执</x:v>
+      </x:c>
+      <x:c r="K21" s="74" t="str">
+        <x:v>https://zqwl-quantum.com/
+https://yxzg.china.com.cn/2026-05/08/content_43421809.shtml</x:v>
+      </x:c>
+      <x:c r="L21" s="77" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="66" customHeight="1">
+      <x:c r="A22" s="75" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B22" s="75" t="str">
+        <x:v>不筹量子</x:v>
+      </x:c>
+      <x:c r="C22" s="75" t="str">
+        <x:v>中性原子</x:v>
+      </x:c>
+      <x:c r="D22" s="74" t="str">
+        <x:v>量筹一号量子 AI 基座及金融、天气、能源算法方案</x:v>
+      </x:c>
+      <x:c r="E22" s="74" t="str">
+        <x:v>中性原子整机、量子云、仪器和智能测控</x:v>
+      </x:c>
+      <x:c r="F22" s="74" t="str">
+        <x:v>已有量子 AI 与自动测控；未见任务拆解和工具调用型 Agent</x:v>
+      </x:c>
+      <x:c r="G22" s="74" t="str">
+        <x:v>公开行为独立实现 + 官方接口接入</x:v>
+      </x:c>
+      <x:c r="H22" s="74" t="str">
+        <x:v>Skill + Tool Provider + Scientific Validator</x:v>
+      </x:c>
+      <x:c r="I22" s="76" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="J22" s="74" t="str">
+        <x:v>核验量筹一号接口、可调用工具、工作流轨迹和客户任务</x:v>
+      </x:c>
+      <x:c r="K22" s="74" t="str">
+        <x:v>https://www.buchouatom.com/</x:v>
+      </x:c>
+      <x:c r="L22" s="77" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="66" customHeight="1">
+      <x:c r="A23" s="75" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B23" s="75" t="str">
+        <x:v>太一量生</x:v>
+      </x:c>
+      <x:c r="C23" s="75" t="str">
+        <x:v>中性原子</x:v>
+      </x:c>
+      <x:c r="D23" s="74" t="str">
+        <x:v>未见公开算法、模拟器或应用服务</x:v>
+      </x:c>
+      <x:c r="E23" s="74" t="str">
+        <x:v>镱原子通用量子计算平台处于早期研发</x:v>
+      </x:c>
+      <x:c r="F23" s="74" t="str">
+        <x:v>未见 Agent</x:v>
+      </x:c>
+      <x:c r="G23" s="74" t="str">
+        <x:v>仅监控</x:v>
+      </x:c>
+      <x:c r="H23" s="74" t="str">
+        <x:v>暂不接入</x:v>
+      </x:c>
+      <x:c r="I23" s="76" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="J23" s="74" t="str">
+        <x:v>等待原型机、软件栈、云/API 和独立官网</x:v>
+      </x:c>
+      <x:c r="K23" s="74" t="str">
+        <x:v>https://vc.pedaily.cn/company/891470.html</x:v>
+      </x:c>
+      <x:c r="L23" s="77" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="66" customHeight="1">
+      <x:c r="A24" s="75" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B24" s="75" t="str">
+        <x:v>纳开科技（纳开量子）</x:v>
+      </x:c>
+      <x:c r="C24" s="75" t="str">
+        <x:v>中性原子</x:v>
+      </x:c>
+      <x:c r="D24" s="74" t="str">
+        <x:v>冷原子与量子模拟实验平台、定制实验和数据服务</x:v>
+      </x:c>
+      <x:c r="E24" s="74" t="str">
+        <x:v>科研仪器、实验模块、定制搭建；未见远程机器接口</x:v>
+      </x:c>
+      <x:c r="F24" s="74" t="str">
+        <x:v>未见 Agent 实验助手</x:v>
+      </x:c>
+      <x:c r="G24" s="74" t="str">
+        <x:v>公开行为独立实现；接口出现后接入</x:v>
+      </x:c>
+      <x:c r="H24" s="74" t="str">
+        <x:v>Skill + Tool Provider + Scientific Validator</x:v>
+      </x:c>
+      <x:c r="I24" s="76" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="J24" s="74" t="str">
+        <x:v>核验远程控制协议、数据格式和实验助手入口</x:v>
+      </x:c>
+      <x:c r="K24" s="74" t="str">
+        <x:v>https://www.nkquantum.com/
+https://www.nkquantum.com/h-pd-21.html</x:v>
+      </x:c>
+      <x:c r="L24" s="77" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="66" customHeight="1">
+      <x:c r="A25" s="75" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B25" s="75" t="str">
+        <x:v>无问清芯</x:v>
+      </x:c>
+      <x:c r="C25" s="75" t="str">
+        <x:v>中性原子</x:v>
+      </x:c>
+      <x:c r="D25" s="74" t="str">
+        <x:v>药物/化学、物流和金融优化的量子算法 SaaS</x:v>
+      </x:c>
+      <x:c r="E25" s="74" t="str">
+        <x:v>算法服务平台；硬件接口和公开 API 尚未确认</x:v>
+      </x:c>
+      <x:c r="F25" s="74" t="str">
+        <x:v>未见任务型 Agent、MCP 或公开 API</x:v>
+      </x:c>
+      <x:c r="G25" s="74" t="str">
+        <x:v>公开行为独立实现；接口出现后接入</x:v>
+      </x:c>
+      <x:c r="H25" s="74" t="str">
+        <x:v>Skill + Tool Provider + Eval</x:v>
+      </x:c>
+      <x:c r="I25" s="76" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="J25" s="74" t="str">
+        <x:v>核验 SaaS 入口、API、运行回执、基准和客户案例</x:v>
+      </x:c>
+      <x:c r="K25" s="74" t="str">
+        <x:v>https://news.pedaily.cn/20260511/129526.shtml
+https://www.jiemian.com/article/14529046.html</x:v>
+      </x:c>
+      <x:c r="L25" s="77" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="66" customHeight="1">
+      <x:c r="A26" s="75" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B26" s="75" t="str">
+        <x:v>原子矩阵</x:v>
+      </x:c>
+      <x:c r="C26" s="75" t="str">
+        <x:v>中性原子</x:v>
+      </x:c>
+      <x:c r="D26" s="74" t="str">
+        <x:v>量子-GPU 混合计算与行业应用方向；公开算法资产未确认</x:v>
+      </x:c>
+      <x:c r="E26" s="74" t="str">
+        <x:v>中性原子整机、全栈系统和 MatriQ 算力云规划</x:v>
+      </x:c>
+      <x:c r="F26" s="74" t="str">
+        <x:v>具备异构调度方向；未见公开 Agent</x:v>
+      </x:c>
+      <x:c r="G26" s="74" t="str">
+        <x:v>公开行为独立实现；未来官方接口接入</x:v>
+      </x:c>
+      <x:c r="H26" s="74" t="str">
+        <x:v>Skill + External API Adapter + Tool Provider</x:v>
+      </x:c>
+      <x:c r="I26" s="76" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="J26" s="74" t="str">
+        <x:v>核验 MatriQ 上线、API、异构调度合同和 Agent 调用</x:v>
+      </x:c>
+      <x:c r="K26" s="74" t="str">
+        <x:v>https://www.puhuacapital.com/mobile/index.php/news/info/327
+https://www.donews.com/news/detail/4/6640575.html</x:v>
+      </x:c>
+      <x:c r="L26" s="77" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="66" customHeight="1">
+      <x:c r="A27" s="75" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B27" s="75" t="str">
+        <x:v>硅臻芯片</x:v>
+      </x:c>
+      <x:c r="C27" s="75" t="str">
+        <x:v>光量子</x:v>
+      </x:c>
+      <x:c r="D27" s="74" t="str">
+        <x:v>可编程光量子实验、QRNG 和教研服务；未确认公开模拟器</x:v>
+      </x:c>
+      <x:c r="E27" s="74" t="str">
+        <x:v>光量子芯片、整机、测控仪器和免费试用入口</x:v>
+      </x:c>
+      <x:c r="F27" s="74" t="str">
+        <x:v>试用入口不等于机器可调用 Agent</x:v>
+      </x:c>
+      <x:c r="G27" s="74" t="str">
+        <x:v>官方接口接入；公开行为独立实现</x:v>
+      </x:c>
+      <x:c r="H27" s="74" t="str">
+        <x:v>External API Adapter + Tool Provider</x:v>
+      </x:c>
+      <x:c r="I27" s="76" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="J27" s="74" t="str">
+        <x:v>核验试用形态、SDK/API、光量子工具和许可证</x:v>
+      </x:c>
+      <x:c r="K27" s="74" t="str">
+        <x:v>https://www.gz-ichip.com/</x:v>
+      </x:c>
+      <x:c r="L27" s="77" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="66" customHeight="1">
+      <x:c r="A28" s="75" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="B28" s="75" t="str">
+        <x:v>玻色量子</x:v>
+      </x:c>
+      <x:c r="C28" s="75" t="str">
+        <x:v>光量子</x:v>
+      </x:c>
+      <x:c r="D28" s="74" t="str">
+        <x:v>Kaiwu SDK、Kaiwu-PyTorch-Plugin、QUBO/组合优化和量子 AI 模型</x:v>
+      </x:c>
+      <x:c r="E28" s="74" t="str">
+        <x:v>相干光量子计算机、量子云枢和行业求解服务</x:v>
+      </x:c>
+      <x:c r="F28" s="74" t="str">
+        <x:v>已有 Agentic QUBO 合作；未确认公司自有端到端 Agent</x:v>
+      </x:c>
+      <x:c r="G28" s="74" t="str">
+        <x:v>Apache-2.0 复用 + 官方接口接入</x:v>
+      </x:c>
+      <x:c r="H28" s="74" t="str">
+        <x:v>Tool Provider + Skill + Eval</x:v>
+      </x:c>
+      <x:c r="I28" s="76" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="J28" s="74" t="str">
+        <x:v>优先评测 KPP 和 QUBO 模板；核验云 API、工具 schema 和执行证据</x:v>
+      </x:c>
+      <x:c r="K28" s="74" t="str">
+        <x:v>https://www.qboson.com/
+https://github.com/qboson
+https://www.qboson.com/about
+https://news.ikanchai.com/2026/0720/663119.shtml</x:v>
+      </x:c>
+      <x:c r="L28" s="77" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="66" customHeight="1">
+      <x:c r="A29" s="75" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B29" s="75" t="str">
+        <x:v>图灵量子</x:v>
+      </x:c>
+      <x:c r="C29" s="75" t="str">
+        <x:v>光量子</x:v>
+      </x:c>
+      <x:c r="D29" s="74" t="str">
+        <x:v>DeepQuantum：光量子、量子机器学习、Fock/Gaussian、张量网络与混合训练</x:v>
+      </x:c>
+      <x:c r="E29" s="74" t="str">
+        <x:v>光量子整机、量擎云、经典-量子混合算力</x:v>
+      </x:c>
+      <x:c r="F29" s="74" t="str">
+        <x:v>QAgent 提供自然语言理解、任务拆解、算法匹配、混合调度和结果生成</x:v>
+      </x:c>
+      <x:c r="G29" s="74" t="str">
+        <x:v>Apache-2.0 复用 + QAgent 公开行为独立实现</x:v>
+      </x:c>
+      <x:c r="H29" s="74" t="str">
+        <x:v>Python MCP Server + Harness MCP Client + Skill + Validator</x:v>
+      </x:c>
+      <x:c r="I29" s="76" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="J29" s="74" t="str">
+        <x:v>先接入小规模 Fock/Gaussian 模拟；再实现 Quantum Job 体验</x:v>
+      </x:c>
+      <x:c r="K29" s="74" t="str">
+        <x:v>https://www.turingq.com/
+https://github.com/TuringQ/deepquantum
+https://www.sh-italent.com/Article/202607/202607230006.shtml</x:v>
+      </x:c>
+      <x:c r="L29" s="77" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="66" customHeight="1">
+      <x:c r="A30" s="75" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B30" s="75" t="str">
+        <x:v>正则量子</x:v>
+      </x:c>
+      <x:c r="C30" s="75" t="str">
+        <x:v>光量子</x:v>
+      </x:c>
+      <x:c r="D30" s="74" t="str">
+        <x:v>光量子计算、探测和信号处理相关软件能力；未确认可复用仓库</x:v>
+      </x:c>
+      <x:c r="E30" s="74" t="str">
+        <x:v>光量子系统、探测器、信号处理与测试协同服务；机器接口未确认</x:v>
+      </x:c>
+      <x:c r="F30" s="74" t="str">
+        <x:v>未见 Agent</x:v>
+      </x:c>
+      <x:c r="G30" s="74" t="str">
+        <x:v>仅监控；接口出现后接入</x:v>
+      </x:c>
+      <x:c r="H30" s="74" t="str">
+        <x:v>暂不接入</x:v>
+      </x:c>
+      <x:c r="I30" s="76" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="J30" s="74" t="str">
+        <x:v>等待 SDK/API、开发者文档、云任务和可验证案例</x:v>
+      </x:c>
+      <x:c r="K30" s="74" t="str">
+        <x:v>https://zzqtech.com/
+https://zzqtech.com/summary</x:v>
+      </x:c>
+      <x:c r="L30" s="77" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="66" customHeight="1">
+      <x:c r="A31" s="75" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B31" s="75" t="str">
+        <x:v>九章量子</x:v>
+      </x:c>
+      <x:c r="C31" s="75" t="str">
+        <x:v>光量子</x:v>
+      </x:c>
+      <x:c r="D31" s="74" t="str">
+        <x:v>光量子算法、科研服务和 AI 量子方向；公开可复用软件未确认</x:v>
+      </x:c>
+      <x:c r="E31" s="74" t="str">
+        <x:v>光量子关键器件、系统和可能的云/平台入口</x:v>
+      </x:c>
+      <x:c r="F31" s="74" t="str">
+        <x:v>存在量子 AI 表述；未见完整任务型 Agent 证据</x:v>
+      </x:c>
+      <x:c r="G31" s="74" t="str">
+        <x:v>公开行为独立实现；接口出现后接入</x:v>
+      </x:c>
+      <x:c r="H31" s="74" t="str">
+        <x:v>Skill + External API Adapter</x:v>
+      </x:c>
+      <x:c r="I31" s="76" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="J31" s="74" t="str">
+        <x:v>核验算法接口、开发者文档、任务回执和 Agent 真实性</x:v>
+      </x:c>
+      <x:c r="K31" s="74" t="str">
+        <x:v>https://www.jiuzhangqt.com/
+https://www.jiuzhangqt.com/company
+https://www.jiuzhangqt.com/products/quantum-computing/jzqai</x:v>
+      </x:c>
+      <x:c r="L31" s="77" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="66" customHeight="1">
+      <x:c r="A32" s="75" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B32" s="75" t="str">
+        <x:v>灵光量子</x:v>
+      </x:c>
+      <x:c r="C32" s="75" t="str">
+        <x:v>光量子</x:v>
+      </x:c>
+      <x:c r="D32" s="74" t="str">
+        <x:v>未确认公开算法、模拟器或 SDK</x:v>
+      </x:c>
+      <x:c r="E32" s="74" t="str">
+        <x:v>光量子科技与产业服务；机器接口未确认</x:v>
+      </x:c>
+      <x:c r="F32" s="74" t="str">
+        <x:v>未见 Agent</x:v>
+      </x:c>
+      <x:c r="G32" s="74" t="str">
+        <x:v>仅监控</x:v>
+      </x:c>
+      <x:c r="H32" s="74" t="str">
+        <x:v>暂不接入</x:v>
+      </x:c>
+      <x:c r="I32" s="76" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="J32" s="74" t="str">
+        <x:v>等待开发者入口、软件仓库、云/API 或 Agent 产品</x:v>
+      </x:c>
+      <x:c r="K32" s="74" t="str">
+        <x:v>https://news.10jqka.com.cn/20260414/c675972226.shtml</x:v>
+      </x:c>
+      <x:c r="L32" s="77" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="66" customHeight="1">
+      <x:c r="A33" s="75" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B33" s="75" t="str">
+        <x:v>国仪量子</x:v>
+      </x:c>
+      <x:c r="C33" s="75" t="str">
+        <x:v>传感/通信延伸</x:v>
+      </x:c>
+      <x:c r="D33" s="74" t="str">
+        <x:v>量子测量、谱仪、传感器数据分析和实验软件能力</x:v>
+      </x:c>
+      <x:c r="E33" s="74" t="str">
+        <x:v>量子仪器、测控设备、芯片与实验平台接口</x:v>
+      </x:c>
+      <x:c r="F33" s="74" t="str">
+        <x:v>可能形成实验 Agent 基础；未见公开完整 Agent</x:v>
+      </x:c>
+      <x:c r="G33" s="74" t="str">
+        <x:v>官方接口接入 + 公开行为独立实现</x:v>
+      </x:c>
+      <x:c r="H33" s="74" t="str">
+        <x:v>Tool Provider + Skill + Scientific Validator</x:v>
+      </x:c>
+      <x:c r="I33" s="76" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="J33" s="74" t="str">
+        <x:v>核验仪器 API、自动分析、实验工作流、远程控制和权限</x:v>
+      </x:c>
+      <x:c r="K33" s="74" t="str">
+        <x:v>https://www.ciqtek.com/
+https://www.ciqtek.com/about.html</x:v>
+      </x:c>
+      <x:c r="L33" s="77" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="66" customHeight="1">
+      <x:c r="A34" s="75" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B34" s="75" t="str">
+        <x:v>问天量子</x:v>
+      </x:c>
+      <x:c r="C34" s="75" t="str">
+        <x:v>传感/通信延伸</x:v>
+      </x:c>
+      <x:c r="D34" s="74" t="str">
+        <x:v>量子安全算法、QKD/QRNG 运维和安全评估能力</x:v>
+      </x:c>
+      <x:c r="E34" s="74" t="str">
+        <x:v>量子安全设备、密钥网络和智能运维平台</x:v>
+      </x:c>
+      <x:c r="F34" s="74" t="str">
+        <x:v>智能运维不自动等于 LLM Agent；未见通用任务 Agent</x:v>
+      </x:c>
+      <x:c r="G34" s="74" t="str">
+        <x:v>官方接口接入 + 公开行为独立实现</x:v>
+      </x:c>
+      <x:c r="H34" s="74" t="str">
+        <x:v>External API Adapter + Tool Provider</x:v>
+      </x:c>
+      <x:c r="I34" s="76" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="J34" s="74" t="str">
+        <x:v>核验设备 API、告警/处置合同、审批边界和审计轨迹</x:v>
+      </x:c>
+      <x:c r="K34" s="74" t="str">
+        <x:v>https://www.qasky.com/
+https://www.qasky.com/wentianliangzi/vip_doc/26917973_0_0_1.html
+https://www.stdaily.com/web/gdxw/2026-08/27/content_570827.html</x:v>
+      </x:c>
+      <x:c r="L34" s="77" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:L1"/>
+    <x:mergeCell ref="A2:L2"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="I5:I34">
+    <x:cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="P0"/>
+    <x:cfRule type="containsText" dxfId="5" priority="2" operator="containsText" text="P1"/>
+    <x:cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="P3"/>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00764a6652414b92"/>
+  </x:tableParts>
+</x:worksheet>
 </file>
</xml_diff>